<commit_message>
Refactor loss coefficient handling: remove global scaling factor and implement per-port loss coefficients in model parameters
</commit_message>
<xml_diff>
--- a/data/examples/3PR-setup.xlsx
+++ b/data/examples/3PR-setup.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="15.33203125" customWidth="1" min="3" max="3"/>
@@ -479,6 +479,16 @@
           <t>Q_setpoint</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>c0</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>c1</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -495,6 +505,12 @@
       <c r="D2" t="n">
         <v>36</v>
       </c>
+      <c r="G2" t="n">
+        <v>-5.82e-05</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.00154</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -511,6 +527,12 @@
       <c r="D3" t="n">
         <v>36</v>
       </c>
+      <c r="G3" t="n">
+        <v>-5.82e-05</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.00154</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -527,6 +549,12 @@
       <c r="D4" t="n">
         <v>36</v>
       </c>
+      <c r="G4" t="n">
+        <v>-5.82e-05</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.00154</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -540,6 +568,12 @@
           <t>slack</t>
         </is>
       </c>
+      <c r="G5" t="n">
+        <v>-5.82e-05</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.00154</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -556,6 +590,12 @@
       <c r="D6" t="n">
         <v>36</v>
       </c>
+      <c r="G6" t="n">
+        <v>-2.328e-05</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.000616</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -569,6 +609,12 @@
           <t>slack</t>
         </is>
       </c>
+      <c r="G7" t="n">
+        <v>-2.328e-05</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.000616</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -582,6 +628,12 @@
           <t>pq</t>
         </is>
       </c>
+      <c r="G8" t="n">
+        <v>-2.328e-05</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.000616</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -603,6 +655,12 @@
       </c>
       <c r="F9" t="n">
         <v>1</v>
+      </c>
+      <c r="G9" t="n">
+        <v>-2.328e-05</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.000616</v>
       </c>
     </row>
   </sheetData>

</xml_diff>